<commit_message>
Fix conflicts by preferring local changes
</commit_message>
<xml_diff>
--- a/data/02_運用_rakuten.xlsx
+++ b/data/02_運用_rakuten.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6ca29965d2a6599a/01_資産管理/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="653" documentId="13_ncr:1_{F23918F6-93A0-4FFC-9C54-3B208A91E086}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CC333871-D026-4D34-B7C9-C8F3DDF947DF}"/>
+  <xr:revisionPtr revIDLastSave="667" documentId="13_ncr:1_{F23918F6-93A0-4FFC-9C54-3B208A91E086}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1B8B5871-07A0-49EA-B826-0AB6072A9C4B}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="819" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7522" uniqueCount="479">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7673" uniqueCount="480">
   <si>
     <t>約定日</t>
   </si>
@@ -2128,6 +2128,9 @@
   <si>
     <t>任天堂</t>
   </si>
+  <si>
+    <t>京都フィナンシャルＧ</t>
+  </si>
 </sst>
 </file>
 
@@ -3430,7 +3433,7 @@
       </c>
       <c r="V2" s="49">
         <f ca="1">TODAY()</f>
-        <v>46199</v>
+        <v>46207</v>
       </c>
     </row>
     <row r="3" spans="1:22" x14ac:dyDescent="0.45">
@@ -3487,31 +3490,31 @@
       </c>
       <c r="D4" s="20">
         <f>SUM(D5:D100)</f>
-        <v>514445</v>
+        <v>519145</v>
       </c>
       <c r="E4" s="35">
         <f>SUM(B4:D4)</f>
-        <v>3177105</v>
+        <v>3181805</v>
       </c>
       <c r="F4" s="20">
         <f>SUM(F5:F100)</f>
-        <v>13664792</v>
+        <v>14015292</v>
       </c>
       <c r="G4" s="20">
         <f>SUM(G5:G100)</f>
-        <v>-5372687</v>
+        <v>-5393677</v>
       </c>
       <c r="H4" s="20">
         <f>SUM(H5:H100)</f>
-        <v>870235</v>
+        <v>916435</v>
       </c>
       <c r="I4" s="35">
         <f>SUM(F4:H4)</f>
-        <v>9162340</v>
+        <v>9538050</v>
       </c>
       <c r="J4" s="35">
         <f>SUM(J5:J100)</f>
-        <v>7301010.6289999997</v>
+        <v>7600395.1425000001</v>
       </c>
       <c r="K4" s="20">
         <f>SUM(K5:K100)</f>
@@ -3519,15 +3522,15 @@
       </c>
       <c r="L4" s="20">
         <f>SUM(L5:L100)</f>
-        <v>-678053</v>
+        <v>-1192189</v>
       </c>
       <c r="M4" s="35">
         <f>SUM(K4:L4)</f>
-        <v>-203805</v>
+        <v>-717941</v>
       </c>
       <c r="N4" s="35">
         <f>SUM(N5:N100)</f>
-        <v>-258697.95835</v>
+        <v>-719996.67485000007</v>
       </c>
       <c r="O4" s="20">
         <f>SUM(O5:O100)</f>
@@ -3547,11 +3550,11 @@
       </c>
       <c r="S4" s="38">
         <f>SUM(E4,J4,N4,R4)</f>
-        <v>10370992.883950001</v>
+        <v>10213778.680950001</v>
       </c>
       <c r="U4" s="56">
         <f ca="1">(V2-U2)/365</f>
-        <v>5.6273972602739724</v>
+        <v>5.6493150684931503</v>
       </c>
       <c r="V4" s="56"/>
     </row>
@@ -3576,11 +3579,11 @@
         <v>160060</v>
       </c>
       <c r="F5" s="19">
-        <f>SUMIFS(国内株式_特定!$N$2:$N$998,国内株式_特定!$B$2:$B$998,"&gt;=2021/1/1",国内株式_特定!$B$2:$B$998,"&lt;=2021/12/31",国内株式_特定!$N$2:$N$998,"&gt;=0")</f>
+        <f>SUMIFS(国内株式_特定!$N$2:$N$996,国内株式_特定!$B$2:$B$996,"&gt;=2021/1/1",国内株式_特定!$B$2:$B$996,"&lt;=2021/12/31",国内株式_特定!$N$2:$N$996,"&gt;=0")</f>
         <v>630746</v>
       </c>
       <c r="G5" s="19">
-        <f>SUMIFS(国内株式_特定!$N$2:$N$998,国内株式_特定!$B$2:$B$998,"&gt;=2021/1/1",国内株式_特定!$B$2:$B$998,"&lt;=2021/12/31",国内株式_特定!$N$2:$N$998,"&lt;0")</f>
+        <f>SUMIFS(国内株式_特定!$N$2:$N$996,国内株式_特定!$B$2:$B$996,"&gt;=2021/1/1",国内株式_特定!$B$2:$B$996,"&lt;=2021/12/31",国内株式_特定!$N$2:$N$996,"&lt;0")</f>
         <v>-601144</v>
       </c>
       <c r="H5" s="19">
@@ -3653,11 +3656,11 @@
         <v>35720</v>
       </c>
       <c r="F6" s="19">
-        <f>SUMIFS(国内株式_特定!$N$2:$N$998,国内株式_特定!$B$2:$B$998,"&gt;=2022/1/1",国内株式_特定!$B$2:$B$998,"&lt;=2022/12/31",国内株式_特定!$N$2:$N$998,"&gt;=0")</f>
+        <f>SUMIFS(国内株式_特定!$N$2:$N$996,国内株式_特定!$B$2:$B$996,"&gt;=2022/1/1",国内株式_特定!$B$2:$B$996,"&lt;=2022/12/31",国内株式_特定!$N$2:$N$996,"&gt;=0")</f>
         <v>619915</v>
       </c>
       <c r="G6" s="19">
-        <f>SUMIFS(国内株式_特定!$N$2:$N$998,国内株式_特定!$B$2:$B$998,"&gt;=2022/1/1",国内株式_特定!$B$2:$B$998,"&lt;=2022/12/31",国内株式_特定!$N$2:$N$998,"&lt;0")</f>
+        <f>SUMIFS(国内株式_特定!$N$2:$N$996,国内株式_特定!$B$2:$B$996,"&gt;=2022/1/1",国内株式_特定!$B$2:$B$996,"&lt;=2022/12/31",国内株式_特定!$N$2:$N$996,"&lt;0")</f>
         <v>-699020</v>
       </c>
       <c r="H6" s="19">
@@ -3730,11 +3733,11 @@
         <v>214320</v>
       </c>
       <c r="F7" s="19">
-        <f>SUMIFS(国内株式_特定!$N$2:$N$998,国内株式_特定!$B$2:$B$998,"&gt;=2023/1/1",国内株式_特定!$B$2:$B$998,"&lt;=2023/12/31",国内株式_特定!$N$2:$N$998,"&gt;=0")</f>
+        <f>SUMIFS(国内株式_特定!$N$2:$N$996,国内株式_特定!$B$2:$B$996,"&gt;=2023/1/1",国内株式_特定!$B$2:$B$996,"&lt;=2023/12/31",国内株式_特定!$N$2:$N$996,"&gt;=0")</f>
         <v>1679057</v>
       </c>
       <c r="G7" s="19">
-        <f>SUMIFS(国内株式_特定!$N$2:$N$998,国内株式_特定!$B$2:$B$998,"&gt;=2023/1/1",国内株式_特定!$B$2:$B$998,"&lt;=2023/12/31",国内株式_特定!$N$2:$N$998,"&lt;0")</f>
+        <f>SUMIFS(国内株式_特定!$N$2:$N$996,国内株式_特定!$B$2:$B$996,"&gt;=2023/1/1",国内株式_特定!$B$2:$B$996,"&lt;=2023/12/31",国内株式_特定!$N$2:$N$996,"&lt;0")</f>
         <v>-402270</v>
       </c>
       <c r="H7" s="19">
@@ -3807,11 +3810,11 @@
         <v>111775</v>
       </c>
       <c r="F8" s="19">
-        <f>SUMIFS(国内株式_特定!$N$2:$N$998,国内株式_特定!$B$2:$B$998,"&gt;=2024/1/1",国内株式_特定!$B$2:$B$998,"&lt;=2024/12/31",国内株式_特定!$N$2:$N$998,"&gt;=0")</f>
+        <f>SUMIFS(国内株式_特定!$N$2:$N$996,国内株式_特定!$B$2:$B$996,"&gt;=2024/1/1",国内株式_特定!$B$2:$B$996,"&lt;=2024/12/31",国内株式_特定!$N$2:$N$996,"&gt;=0")</f>
         <v>2059210</v>
       </c>
       <c r="G8" s="19">
-        <f>SUMIFS(国内株式_特定!$N$2:$N$998,国内株式_特定!$B$2:$B$998,"&gt;=2024/1/1",国内株式_特定!$B$2:$B$998,"&lt;=2024/12/31",国内株式_特定!$N$2:$N$998,"&lt;0")</f>
+        <f>SUMIFS(国内株式_特定!$N$2:$N$996,国内株式_特定!$B$2:$B$996,"&gt;=2024/1/1",国内株式_特定!$B$2:$B$996,"&lt;=2024/12/31",国内株式_特定!$N$2:$N$996,"&lt;0")</f>
         <v>-1123620</v>
       </c>
       <c r="H8" s="19">
@@ -3884,11 +3887,11 @@
         <v>2647720</v>
       </c>
       <c r="F9" s="19">
-        <f>SUMIFS(国内株式_特定!$N$2:$N$998,国内株式_特定!$B$2:$B$998,"&gt;=2025/1/1",国内株式_特定!$B$2:$B$998,"&lt;=2025/12/31",国内株式_特定!$N$2:$N$998,"&gt;=0")</f>
+        <f>SUMIFS(国内株式_特定!$N$2:$N$996,国内株式_特定!$B$2:$B$996,"&gt;=2025/1/1",国内株式_特定!$B$2:$B$996,"&lt;=2025/12/31",国内株式_特定!$N$2:$N$996,"&gt;=0")</f>
         <v>2657465</v>
       </c>
       <c r="G9" s="19">
-        <f>SUMIFS(国内株式_特定!$N$2:$N$998,国内株式_特定!$B$2:$B$998,"&gt;=2025/1/1",国内株式_特定!$B$2:$B$998,"&lt;=2025/12/31",国内株式_特定!$N$2:$N$998,"&lt;0")</f>
+        <f>SUMIFS(国内株式_特定!$N$2:$N$996,国内株式_特定!$B$2:$B$996,"&gt;=2025/1/1",国内株式_特定!$B$2:$B$996,"&lt;=2025/12/31",国内株式_特定!$N$2:$N$996,"&lt;0")</f>
         <v>-599245</v>
       </c>
       <c r="H9" s="19">
@@ -3954,31 +3957,31 @@
       </c>
       <c r="D10" s="19">
         <f>SUMIFS(国内株式_NISA_配当!$K$2:$K$1004,国内株式_NISA_配当!$A$2:$A$1004,"&gt;=2026/1/1",国内株式_NISA_配当!$A$2:$A$1004,"&lt;=2026/12/31")</f>
-        <v>64150</v>
+        <v>68850</v>
       </c>
       <c r="E10" s="35">
         <f t="shared" si="7"/>
-        <v>7510</v>
+        <v>12210</v>
       </c>
       <c r="F10" s="19">
-        <f>SUMIFS(国内株式_特定!$N$2:$N$998,国内株式_特定!$B$2:$B$998,"&gt;=2026/1/1",国内株式_特定!$B$2:$B$998,"&lt;=2026/12/31",国内株式_特定!$N$2:$N$998,"&gt;=0")</f>
-        <v>6018399</v>
+        <f>SUMIFS(国内株式_特定!$N$2:$N$996,国内株式_特定!$B$2:$B$996,"&gt;=2026/1/1",国内株式_特定!$B$2:$B$996,"&lt;=2026/12/31",国内株式_特定!$N$2:$N$996,"&gt;=0")</f>
+        <v>6368899</v>
       </c>
       <c r="G10" s="19">
-        <f>SUMIFS(国内株式_特定!$N$2:$N$998,国内株式_特定!$B$2:$B$998,"&gt;=2026/1/1",国内株式_特定!$B$2:$B$998,"&lt;=2026/12/31",国内株式_特定!$N$2:$N$998,"&lt;0")</f>
-        <v>-1947388</v>
+        <f>SUMIFS(国内株式_特定!$N$2:$N$996,国内株式_特定!$B$2:$B$996,"&gt;=2026/1/1",国内株式_特定!$B$2:$B$996,"&lt;=2026/12/31",国内株式_特定!$N$2:$N$996,"&lt;0")</f>
+        <v>-1968378</v>
       </c>
       <c r="H10" s="19">
         <f>SUMIFS(国内株式_特定_配当!$H$2:$H$999,国内株式_特定_配当!$A$2:$A$999,"&gt;=2026/1/1",国内株式_特定_配当!$A$2:$A$999,"&lt;=2026/12/31")</f>
-        <v>68080</v>
+        <v>114280</v>
       </c>
       <c r="I10" s="35">
         <f t="shared" si="11"/>
-        <v>4139091</v>
+        <v>4514801</v>
       </c>
       <c r="J10" s="36">
         <f t="shared" si="1"/>
-        <v>3298234.66335</v>
+        <v>3597619.1768499999</v>
       </c>
       <c r="K10" s="19">
         <f>SUMIFS(国内株式_信用!$P$2:$P$1000,国内株式_信用!$B$2:$B$1000,"&gt;=2026/1/1",国内株式_信用!$B$2:$B$1000,"&lt;=2026/12/31",国内株式_信用!$P$2:$P$1000,"&gt;=0")</f>
@@ -3986,15 +3989,15 @@
       </c>
       <c r="L10" s="19">
         <f>SUMIFS(国内株式_信用!$P$2:$P$1000,国内株式_信用!$B$2:$B$1000,"&gt;=2026/1/1",国内株式_信用!$B$2:$B$1000,"&lt;=2026/12/31",国内株式_信用!$P$2:$P$1000,"&lt;0")</f>
-        <v>-3810</v>
+        <v>-517946</v>
       </c>
       <c r="M10" s="35">
         <f t="shared" si="12"/>
-        <v>260090</v>
+        <v>-254046</v>
       </c>
       <c r="N10" s="36">
         <f t="shared" si="13"/>
-        <v>207252.71650000001</v>
+        <v>-254046</v>
       </c>
       <c r="O10" s="19">
         <f>SUMIFS(投資信託!$K$2:$K$1033,投資信託!$B$2:$B$1033,"&gt;=2026/1/1",投資信託!$B$2:$B$1033,"&lt;=2026/12/31",投資信託!$K$2:$K$1033,"&gt;=0")</f>
@@ -4014,7 +4017,7 @@
       </c>
       <c r="S10" s="38">
         <f>SUM(E10,J10,N10,R10)</f>
-        <v>3512997.3798500001</v>
+        <v>3355783.1768499999</v>
       </c>
     </row>
     <row r="16" spans="1:22" x14ac:dyDescent="0.45">
@@ -10112,7 +10115,7 @@
   <sheetPr>
     <tabColor theme="7" tint="0.79998168889431442"/>
   </sheetPr>
-  <dimension ref="A1:K67"/>
+  <dimension ref="A1:K68"/>
   <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="11.19921875" style="1" bestFit="1" customWidth="1"/>
@@ -12540,18 +12543,18 @@
         <v>100</v>
       </c>
       <c r="H64" s="19">
-        <f t="shared" ref="H64:H67" si="6">F64*G64</f>
+        <f t="shared" ref="H64:H68" si="6">F64*G64</f>
         <v>4000</v>
       </c>
       <c r="I64" s="19">
         <v>0</v>
       </c>
       <c r="J64" s="19">
-        <f t="shared" ref="J64:J67" si="7">H64-I64</f>
+        <f t="shared" ref="J64:J68" si="7">H64-I64</f>
         <v>4000</v>
       </c>
       <c r="K64" s="19">
-        <f t="shared" ref="K64:K67" si="8">J64</f>
+        <f t="shared" ref="K64:K68" si="8">J64</f>
         <v>4000</v>
       </c>
     </row>
@@ -12667,6 +12670,44 @@
       <c r="K67" s="19">
         <f t="shared" si="8"/>
         <v>10000</v>
+      </c>
+    </row>
+    <row r="68" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A68" s="4">
+        <v>46203</v>
+      </c>
+      <c r="B68" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="C68" s="5" t="s">
+        <v>257</v>
+      </c>
+      <c r="D68" s="5">
+        <v>1802</v>
+      </c>
+      <c r="E68" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="F68" s="23">
+        <v>47</v>
+      </c>
+      <c r="G68" s="5">
+        <v>100</v>
+      </c>
+      <c r="H68" s="19">
+        <f t="shared" si="6"/>
+        <v>4700</v>
+      </c>
+      <c r="I68" s="19">
+        <v>0</v>
+      </c>
+      <c r="J68" s="19">
+        <f t="shared" si="7"/>
+        <v>4700</v>
+      </c>
+      <c r="K68" s="19">
+        <f t="shared" si="8"/>
+        <v>4700</v>
       </c>
     </row>
   </sheetData>
@@ -12686,7 +12727,7 @@
   <sheetPr>
     <tabColor theme="8" tint="0.79998168889431442"/>
   </sheetPr>
-  <dimension ref="A1:O981"/>
+  <dimension ref="A1:O992"/>
   <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="2" width="12.59765625" style="1" bestFit="1" customWidth="1"/>
@@ -54904,7 +54945,7 @@
         <v>31</v>
       </c>
       <c r="M938" s="15">
-        <f t="shared" ref="M938:M981" si="21">IF(G938="買付",H938*I938+SUM(J938:K938),H938*I938-SUM(J938:K938))</f>
+        <f t="shared" ref="M938:M992" si="21">IF(G938="買付",H938*I938+SUM(J938:K938),H938*I938-SUM(J938:K938))</f>
         <v>526900</v>
       </c>
       <c r="N938" s="19">
@@ -56845,6 +56886,501 @@
       </c>
       <c r="N981" s="19">
         <v>0</v>
+      </c>
+    </row>
+    <row r="982" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A982" s="4">
+        <v>46202</v>
+      </c>
+      <c r="B982" s="4">
+        <v>46204</v>
+      </c>
+      <c r="C982" s="5">
+        <v>5844</v>
+      </c>
+      <c r="D982" s="9" t="s">
+        <v>479</v>
+      </c>
+      <c r="E982" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="F982" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G982" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="H982" s="5">
+        <v>100</v>
+      </c>
+      <c r="I982" s="7">
+        <v>4496.5</v>
+      </c>
+      <c r="J982" s="9">
+        <v>0</v>
+      </c>
+      <c r="K982" s="9">
+        <v>0</v>
+      </c>
+      <c r="L982" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="M982" s="15">
+        <f t="shared" si="21"/>
+        <v>449650</v>
+      </c>
+      <c r="N982" s="19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="983" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A983" s="4">
+        <v>46202</v>
+      </c>
+      <c r="B983" s="4">
+        <v>46204</v>
+      </c>
+      <c r="C983" s="5">
+        <v>6324</v>
+      </c>
+      <c r="D983" s="9" t="s">
+        <v>454</v>
+      </c>
+      <c r="E983" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="F983" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G983" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="H983" s="5">
+        <v>100</v>
+      </c>
+      <c r="I983" s="7">
+        <v>7120</v>
+      </c>
+      <c r="J983" s="9">
+        <v>0</v>
+      </c>
+      <c r="K983" s="9">
+        <v>0</v>
+      </c>
+      <c r="L983" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="M983" s="15">
+        <f t="shared" si="21"/>
+        <v>712000</v>
+      </c>
+      <c r="N983" s="19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="984" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A984" s="4">
+        <v>46202</v>
+      </c>
+      <c r="B984" s="4">
+        <v>46204</v>
+      </c>
+      <c r="C984" s="5">
+        <v>6857</v>
+      </c>
+      <c r="D984" s="9" t="s">
+        <v>458</v>
+      </c>
+      <c r="E984" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="F984" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G984" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="H984" s="5">
+        <v>100</v>
+      </c>
+      <c r="I984" s="7">
+        <v>31960</v>
+      </c>
+      <c r="J984" s="9">
+        <v>0</v>
+      </c>
+      <c r="K984" s="9">
+        <v>0</v>
+      </c>
+      <c r="L984" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="M984" s="15">
+        <f t="shared" si="21"/>
+        <v>3196000</v>
+      </c>
+      <c r="N984" s="19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="985" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A985" s="4">
+        <v>46203</v>
+      </c>
+      <c r="B985" s="4">
+        <v>46205</v>
+      </c>
+      <c r="C985" s="5">
+        <v>6857</v>
+      </c>
+      <c r="D985" s="9" t="s">
+        <v>458</v>
+      </c>
+      <c r="E985" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="F985" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G985" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="H985" s="5">
+        <v>100</v>
+      </c>
+      <c r="I985" s="7">
+        <v>31750.1</v>
+      </c>
+      <c r="J985" s="9">
+        <v>0</v>
+      </c>
+      <c r="K985" s="9">
+        <v>0</v>
+      </c>
+      <c r="L985" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="M985" s="15">
+        <f t="shared" si="21"/>
+        <v>3175010</v>
+      </c>
+      <c r="N985" s="19">
+        <v>-20990</v>
+      </c>
+    </row>
+    <row r="986" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A986" s="4">
+        <v>46203</v>
+      </c>
+      <c r="B986" s="4">
+        <v>46205</v>
+      </c>
+      <c r="C986" s="5">
+        <v>6324</v>
+      </c>
+      <c r="D986" s="9" t="s">
+        <v>454</v>
+      </c>
+      <c r="E986" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="F986" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G986" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="H986" s="5">
+        <v>100</v>
+      </c>
+      <c r="I986" s="7">
+        <v>7295</v>
+      </c>
+      <c r="J986" s="9">
+        <v>0</v>
+      </c>
+      <c r="K986" s="9">
+        <v>0</v>
+      </c>
+      <c r="L986" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="M986" s="15">
+        <f t="shared" si="21"/>
+        <v>729500</v>
+      </c>
+      <c r="N986" s="19">
+        <v>17500</v>
+      </c>
+    </row>
+    <row r="987" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A987" s="4">
+        <v>46203</v>
+      </c>
+      <c r="B987" s="4">
+        <v>46205</v>
+      </c>
+      <c r="C987" s="5" t="s">
+        <v>446</v>
+      </c>
+      <c r="D987" s="9" t="s">
+        <v>447</v>
+      </c>
+      <c r="E987" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="F987" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G987" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="H987" s="5">
+        <v>100</v>
+      </c>
+      <c r="I987" s="7">
+        <v>91050</v>
+      </c>
+      <c r="J987" s="9">
+        <v>0</v>
+      </c>
+      <c r="K987" s="9">
+        <v>0</v>
+      </c>
+      <c r="L987" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="M987" s="15">
+        <f t="shared" si="21"/>
+        <v>9105000</v>
+      </c>
+      <c r="N987" s="19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="988" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A988" s="4">
+        <v>46203</v>
+      </c>
+      <c r="B988" s="4">
+        <v>46205</v>
+      </c>
+      <c r="C988" s="5" t="s">
+        <v>446</v>
+      </c>
+      <c r="D988" s="9" t="s">
+        <v>447</v>
+      </c>
+      <c r="E988" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="F988" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G988" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="H988" s="5">
+        <v>100</v>
+      </c>
+      <c r="I988" s="7">
+        <v>91660</v>
+      </c>
+      <c r="J988" s="9">
+        <v>0</v>
+      </c>
+      <c r="K988" s="9">
+        <v>0</v>
+      </c>
+      <c r="L988" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="M988" s="15">
+        <f t="shared" si="21"/>
+        <v>9166000</v>
+      </c>
+      <c r="N988" s="19">
+        <v>61000</v>
+      </c>
+    </row>
+    <row r="989" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A989" s="4">
+        <v>46205</v>
+      </c>
+      <c r="B989" s="4">
+        <v>46209</v>
+      </c>
+      <c r="C989" s="5">
+        <v>5844</v>
+      </c>
+      <c r="D989" s="9" t="s">
+        <v>479</v>
+      </c>
+      <c r="E989" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="F989" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G989" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="H989" s="5">
+        <v>100</v>
+      </c>
+      <c r="I989" s="7">
+        <v>4653</v>
+      </c>
+      <c r="J989" s="9">
+        <v>0</v>
+      </c>
+      <c r="K989" s="9">
+        <v>0</v>
+      </c>
+      <c r="L989" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="M989" s="15">
+        <f t="shared" si="21"/>
+        <v>465300</v>
+      </c>
+      <c r="N989" s="19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="990" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A990" s="4">
+        <v>46205</v>
+      </c>
+      <c r="B990" s="4">
+        <v>46209</v>
+      </c>
+      <c r="C990" s="5">
+        <v>8766</v>
+      </c>
+      <c r="D990" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="E990" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="F990" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G990" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="H990" s="5">
+        <v>100</v>
+      </c>
+      <c r="I990" s="7">
+        <v>7479.9</v>
+      </c>
+      <c r="J990" s="9">
+        <v>0</v>
+      </c>
+      <c r="K990" s="9">
+        <v>0</v>
+      </c>
+      <c r="L990" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="M990" s="15">
+        <f t="shared" si="21"/>
+        <v>747990</v>
+      </c>
+      <c r="N990" s="19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="991" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A991" s="4">
+        <v>46206</v>
+      </c>
+      <c r="B991" s="4">
+        <v>46210</v>
+      </c>
+      <c r="C991" s="5" t="s">
+        <v>446</v>
+      </c>
+      <c r="D991" s="9" t="s">
+        <v>447</v>
+      </c>
+      <c r="E991" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="F991" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G991" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="H991" s="5">
+        <v>100</v>
+      </c>
+      <c r="I991" s="7">
+        <v>79080</v>
+      </c>
+      <c r="J991" s="9">
+        <v>0</v>
+      </c>
+      <c r="K991" s="9">
+        <v>0</v>
+      </c>
+      <c r="L991" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="M991" s="15">
+        <f t="shared" si="21"/>
+        <v>7908000</v>
+      </c>
+      <c r="N991" s="19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="992" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A992" s="4">
+        <v>46206</v>
+      </c>
+      <c r="B992" s="4">
+        <v>46210</v>
+      </c>
+      <c r="C992" s="5" t="s">
+        <v>446</v>
+      </c>
+      <c r="D992" s="9" t="s">
+        <v>447</v>
+      </c>
+      <c r="E992" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="F992" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G992" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="H992" s="5">
+        <v>100</v>
+      </c>
+      <c r="I992" s="7">
+        <v>81800</v>
+      </c>
+      <c r="J992" s="9">
+        <v>0</v>
+      </c>
+      <c r="K992" s="9">
+        <v>0</v>
+      </c>
+      <c r="L992" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="M992" s="15">
+        <f t="shared" si="21"/>
+        <v>8180000</v>
+      </c>
+      <c r="N992" s="19">
+        <v>272000</v>
       </c>
     </row>
   </sheetData>
@@ -56864,7 +57400,7 @@
   <sheetPr>
     <tabColor theme="8" tint="0.79998168889431442"/>
   </sheetPr>
-  <dimension ref="A1:M97"/>
+  <dimension ref="A1:M104"/>
   <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="11.19921875" style="1" bestFit="1" customWidth="1"/>
@@ -60169,7 +60705,7 @@
         <v>100</v>
       </c>
       <c r="H87" s="19">
-        <f t="shared" ref="H87:H97" si="18">F87*G87</f>
+        <f t="shared" ref="H87:H104" si="18">F87*G87</f>
         <v>8000</v>
       </c>
       <c r="I87" s="19">
@@ -60480,11 +61016,11 @@
         <v>240</v>
       </c>
       <c r="J95" s="19">
-        <f t="shared" ref="J95:J97" si="19">H95-I95</f>
+        <f t="shared" ref="J95:J104" si="19">H95-I95</f>
         <v>945</v>
       </c>
       <c r="K95" s="19">
-        <f t="shared" ref="K95:K97" si="20">J95</f>
+        <f t="shared" ref="K95:K104" si="20">J95</f>
         <v>945</v>
       </c>
     </row>
@@ -60562,6 +61098,272 @@
       <c r="K97" s="19">
         <f t="shared" si="20"/>
         <v>7650</v>
+      </c>
+    </row>
+    <row r="98" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A98" s="4">
+        <v>46202</v>
+      </c>
+      <c r="B98" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="C98" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="D98" s="5">
+        <v>7974</v>
+      </c>
+      <c r="E98" s="9" t="s">
+        <v>174</v>
+      </c>
+      <c r="F98" s="9">
+        <v>177</v>
+      </c>
+      <c r="G98" s="5">
+        <v>100</v>
+      </c>
+      <c r="H98" s="19">
+        <f t="shared" si="18"/>
+        <v>17700</v>
+      </c>
+      <c r="I98" s="19">
+        <v>3595</v>
+      </c>
+      <c r="J98" s="19">
+        <f t="shared" si="19"/>
+        <v>14105</v>
+      </c>
+      <c r="K98" s="19">
+        <f t="shared" si="20"/>
+        <v>14105</v>
+      </c>
+    </row>
+    <row r="99" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A99" s="4">
+        <v>46202</v>
+      </c>
+      <c r="B99" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="C99" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="D99" s="5">
+        <v>7011</v>
+      </c>
+      <c r="E99" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="F99" s="9">
+        <v>13</v>
+      </c>
+      <c r="G99" s="5">
+        <v>500</v>
+      </c>
+      <c r="H99" s="19">
+        <f t="shared" si="18"/>
+        <v>6500</v>
+      </c>
+      <c r="I99" s="19">
+        <v>1320</v>
+      </c>
+      <c r="J99" s="19">
+        <f t="shared" si="19"/>
+        <v>5180</v>
+      </c>
+      <c r="K99" s="19">
+        <f t="shared" si="20"/>
+        <v>5180</v>
+      </c>
+    </row>
+    <row r="100" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A100" s="4">
+        <v>46202</v>
+      </c>
+      <c r="B100" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="C100" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="D100" s="5">
+        <v>7003</v>
+      </c>
+      <c r="E100" s="9" t="s">
+        <v>444</v>
+      </c>
+      <c r="F100" s="9">
+        <v>42</v>
+      </c>
+      <c r="G100" s="5">
+        <v>100</v>
+      </c>
+      <c r="H100" s="19">
+        <f t="shared" si="18"/>
+        <v>4200</v>
+      </c>
+      <c r="I100" s="19">
+        <v>853</v>
+      </c>
+      <c r="J100" s="19">
+        <f t="shared" si="19"/>
+        <v>3347</v>
+      </c>
+      <c r="K100" s="19">
+        <f t="shared" si="20"/>
+        <v>3347</v>
+      </c>
+    </row>
+    <row r="101" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A101" s="4">
+        <v>46202</v>
+      </c>
+      <c r="B101" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="C101" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="D101" s="5">
+        <v>5016</v>
+      </c>
+      <c r="E101" s="9" t="s">
+        <v>439</v>
+      </c>
+      <c r="F101" s="9">
+        <v>25</v>
+      </c>
+      <c r="G101" s="5">
+        <v>100</v>
+      </c>
+      <c r="H101" s="19">
+        <f t="shared" si="18"/>
+        <v>2500</v>
+      </c>
+      <c r="I101" s="19">
+        <v>507</v>
+      </c>
+      <c r="J101" s="19">
+        <f t="shared" si="19"/>
+        <v>1993</v>
+      </c>
+      <c r="K101" s="19">
+        <f t="shared" si="20"/>
+        <v>1993</v>
+      </c>
+    </row>
+    <row r="102" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A102" s="4">
+        <v>46202</v>
+      </c>
+      <c r="B102" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="C102" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="D102" s="5">
+        <v>4661</v>
+      </c>
+      <c r="E102" s="9" t="s">
+        <v>220</v>
+      </c>
+      <c r="F102" s="9">
+        <v>8</v>
+      </c>
+      <c r="G102" s="5">
+        <v>100</v>
+      </c>
+      <c r="H102" s="19">
+        <f t="shared" si="18"/>
+        <v>800</v>
+      </c>
+      <c r="I102" s="19">
+        <v>162</v>
+      </c>
+      <c r="J102" s="19">
+        <f t="shared" si="19"/>
+        <v>638</v>
+      </c>
+      <c r="K102" s="19">
+        <f t="shared" si="20"/>
+        <v>638</v>
+      </c>
+    </row>
+    <row r="103" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A103" s="4">
+        <v>46202</v>
+      </c>
+      <c r="B103" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="C103" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="D103" s="5">
+        <v>2201</v>
+      </c>
+      <c r="E103" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="F103" s="9">
+        <v>32.5</v>
+      </c>
+      <c r="G103" s="5">
+        <v>100</v>
+      </c>
+      <c r="H103" s="19">
+        <f t="shared" si="18"/>
+        <v>3250</v>
+      </c>
+      <c r="I103" s="19">
+        <v>659</v>
+      </c>
+      <c r="J103" s="19">
+        <f t="shared" si="19"/>
+        <v>2591</v>
+      </c>
+      <c r="K103" s="19">
+        <f t="shared" si="20"/>
+        <v>2591</v>
+      </c>
+    </row>
+    <row r="104" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A104" s="4">
+        <v>46203</v>
+      </c>
+      <c r="B104" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="C104" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="D104" s="5">
+        <v>8766</v>
+      </c>
+      <c r="E104" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="F104" s="9">
+        <v>112.5</v>
+      </c>
+      <c r="G104" s="5">
+        <v>100</v>
+      </c>
+      <c r="H104" s="19">
+        <f t="shared" si="18"/>
+        <v>11250</v>
+      </c>
+      <c r="I104" s="19">
+        <v>2284</v>
+      </c>
+      <c r="J104" s="19">
+        <f t="shared" si="19"/>
+        <v>8966</v>
+      </c>
+      <c r="K104" s="19">
+        <f t="shared" si="20"/>
+        <v>8966</v>
       </c>
     </row>
   </sheetData>
@@ -60577,7 +61379,7 @@
   <sheetPr>
     <tabColor theme="4" tint="0.79998168889431442"/>
   </sheetPr>
-  <dimension ref="A1:AA77"/>
+  <dimension ref="A1:AA85"/>
   <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="2" width="11.296875" style="1" bestFit="1" customWidth="1"/>
@@ -66318,7 +67120,7 @@
       <c r="P70" s="8">
         <v>18867</v>
       </c>
-      <c r="Q70" s="49">
+      <c r="Q70" s="4">
         <v>46091</v>
       </c>
       <c r="R70" s="7">
@@ -66401,7 +67203,7 @@
       <c r="P71" s="9">
         <v>0</v>
       </c>
-      <c r="Q71" s="9" t="s">
+      <c r="Q71" s="6" t="s">
         <v>31</v>
       </c>
       <c r="R71" s="9">
@@ -66484,7 +67286,7 @@
       <c r="P72" s="8">
         <v>39427</v>
       </c>
-      <c r="Q72" s="49">
+      <c r="Q72" s="4">
         <v>46091</v>
       </c>
       <c r="R72" s="7">
@@ -66567,7 +67369,7 @@
       <c r="P73" s="9">
         <v>0</v>
       </c>
-      <c r="Q73" s="9" t="s">
+      <c r="Q73" s="6" t="s">
         <v>31</v>
       </c>
       <c r="R73" s="9">
@@ -66650,7 +67452,7 @@
       <c r="P74" s="8">
         <v>46089</v>
       </c>
-      <c r="Q74" s="49">
+      <c r="Q74" s="4">
         <v>46091</v>
       </c>
       <c r="R74" s="7">
@@ -66733,7 +67535,7 @@
       <c r="P75" s="9">
         <v>0</v>
       </c>
-      <c r="Q75" s="9" t="s">
+      <c r="Q75" s="6" t="s">
         <v>31</v>
       </c>
       <c r="R75" s="9">
@@ -66928,6 +67730,666 @@
         <v>0</v>
       </c>
       <c r="AA77" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78" spans="1:27" x14ac:dyDescent="0.45">
+      <c r="A78" s="4">
+        <v>46202</v>
+      </c>
+      <c r="B78" s="4">
+        <v>46204</v>
+      </c>
+      <c r="C78" s="5" t="s">
+        <v>446</v>
+      </c>
+      <c r="D78" s="9" t="s">
+        <v>447</v>
+      </c>
+      <c r="E78" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="F78" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="G78" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="H78" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="I78" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="J78" s="5">
+        <v>100</v>
+      </c>
+      <c r="K78" s="7">
+        <v>86800</v>
+      </c>
+      <c r="L78" s="9">
+        <v>0</v>
+      </c>
+      <c r="M78" s="9">
+        <v>0</v>
+      </c>
+      <c r="N78" s="9">
+        <v>257</v>
+      </c>
+      <c r="O78" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="P78" s="20">
+        <v>-120257</v>
+      </c>
+      <c r="Q78" s="4">
+        <v>46202</v>
+      </c>
+      <c r="R78" s="7">
+        <v>85600</v>
+      </c>
+      <c r="S78" s="9">
+        <v>0</v>
+      </c>
+      <c r="T78" s="9">
+        <v>0</v>
+      </c>
+      <c r="U78" s="9">
+        <v>0</v>
+      </c>
+      <c r="V78" s="9">
+        <v>0</v>
+      </c>
+      <c r="W78" s="9">
+        <v>0</v>
+      </c>
+      <c r="X78" s="9">
+        <v>0</v>
+      </c>
+      <c r="Y78" s="9">
+        <v>257</v>
+      </c>
+      <c r="Z78" s="9">
+        <v>0</v>
+      </c>
+      <c r="AA78" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79" spans="1:27" x14ac:dyDescent="0.45">
+      <c r="A79" s="4">
+        <v>46202</v>
+      </c>
+      <c r="B79" s="4">
+        <v>46204</v>
+      </c>
+      <c r="C79" s="5" t="s">
+        <v>446</v>
+      </c>
+      <c r="D79" s="9" t="s">
+        <v>447</v>
+      </c>
+      <c r="E79" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="F79" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="G79" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="H79" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="I79" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="J79" s="5">
+        <v>100</v>
+      </c>
+      <c r="K79" s="7">
+        <v>85600</v>
+      </c>
+      <c r="L79" s="9">
+        <v>0</v>
+      </c>
+      <c r="M79" s="9">
+        <v>0</v>
+      </c>
+      <c r="N79" s="9">
+        <v>0</v>
+      </c>
+      <c r="O79" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="P79" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q79" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="R79" s="9">
+        <v>0</v>
+      </c>
+      <c r="S79" s="9">
+        <v>0</v>
+      </c>
+      <c r="T79" s="9">
+        <v>0</v>
+      </c>
+      <c r="U79" s="9">
+        <v>0</v>
+      </c>
+      <c r="V79" s="9">
+        <v>0</v>
+      </c>
+      <c r="W79" s="9">
+        <v>0</v>
+      </c>
+      <c r="X79" s="9">
+        <v>0</v>
+      </c>
+      <c r="Y79" s="9">
+        <v>0</v>
+      </c>
+      <c r="Z79" s="9">
+        <v>0</v>
+      </c>
+      <c r="AA79" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80" spans="1:27" x14ac:dyDescent="0.45">
+      <c r="A80" s="4">
+        <v>46202</v>
+      </c>
+      <c r="B80" s="4">
+        <v>46204</v>
+      </c>
+      <c r="C80" s="5">
+        <v>6857</v>
+      </c>
+      <c r="D80" s="9" t="s">
+        <v>458</v>
+      </c>
+      <c r="E80" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="F80" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="G80" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="H80" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="I80" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="J80" s="5">
+        <v>100</v>
+      </c>
+      <c r="K80" s="7">
+        <v>31710</v>
+      </c>
+      <c r="L80" s="9">
+        <v>0</v>
+      </c>
+      <c r="M80" s="9">
+        <v>0</v>
+      </c>
+      <c r="N80" s="9">
+        <v>94</v>
+      </c>
+      <c r="O80" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="P80" s="20">
+        <v>-46094</v>
+      </c>
+      <c r="Q80" s="4">
+        <v>46202</v>
+      </c>
+      <c r="R80" s="7">
+        <v>31250</v>
+      </c>
+      <c r="S80" s="9">
+        <v>0</v>
+      </c>
+      <c r="T80" s="9">
+        <v>0</v>
+      </c>
+      <c r="U80" s="9">
+        <v>0</v>
+      </c>
+      <c r="V80" s="9">
+        <v>0</v>
+      </c>
+      <c r="W80" s="9">
+        <v>0</v>
+      </c>
+      <c r="X80" s="9">
+        <v>0</v>
+      </c>
+      <c r="Y80" s="9">
+        <v>94</v>
+      </c>
+      <c r="Z80" s="9">
+        <v>0</v>
+      </c>
+      <c r="AA80" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81" spans="1:27" x14ac:dyDescent="0.45">
+      <c r="A81" s="4">
+        <v>46202</v>
+      </c>
+      <c r="B81" s="4">
+        <v>46204</v>
+      </c>
+      <c r="C81" s="5">
+        <v>6857</v>
+      </c>
+      <c r="D81" s="9" t="s">
+        <v>458</v>
+      </c>
+      <c r="E81" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="F81" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="G81" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="H81" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="I81" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="J81" s="5">
+        <v>100</v>
+      </c>
+      <c r="K81" s="7">
+        <v>31250</v>
+      </c>
+      <c r="L81" s="9">
+        <v>0</v>
+      </c>
+      <c r="M81" s="9">
+        <v>0</v>
+      </c>
+      <c r="N81" s="9">
+        <v>0</v>
+      </c>
+      <c r="O81" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="P81" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q81" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="R81" s="9">
+        <v>0</v>
+      </c>
+      <c r="S81" s="9">
+        <v>0</v>
+      </c>
+      <c r="T81" s="9">
+        <v>0</v>
+      </c>
+      <c r="U81" s="9">
+        <v>0</v>
+      </c>
+      <c r="V81" s="9">
+        <v>0</v>
+      </c>
+      <c r="W81" s="9">
+        <v>0</v>
+      </c>
+      <c r="X81" s="9">
+        <v>0</v>
+      </c>
+      <c r="Y81" s="9">
+        <v>0</v>
+      </c>
+      <c r="Z81" s="9">
+        <v>0</v>
+      </c>
+      <c r="AA81" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82" spans="1:27" x14ac:dyDescent="0.45">
+      <c r="A82" s="4">
+        <v>46203</v>
+      </c>
+      <c r="B82" s="4">
+        <v>46205</v>
+      </c>
+      <c r="C82" s="5">
+        <v>6857</v>
+      </c>
+      <c r="D82" s="9" t="s">
+        <v>458</v>
+      </c>
+      <c r="E82" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="F82" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="G82" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="H82" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="I82" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="J82" s="5">
+        <v>100</v>
+      </c>
+      <c r="K82" s="7">
+        <v>31600</v>
+      </c>
+      <c r="L82" s="9">
+        <v>0</v>
+      </c>
+      <c r="M82" s="9">
+        <v>0</v>
+      </c>
+      <c r="N82" s="9">
+        <v>0</v>
+      </c>
+      <c r="O82" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="P82" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q82" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="R82" s="9">
+        <v>0</v>
+      </c>
+      <c r="S82" s="9">
+        <v>0</v>
+      </c>
+      <c r="T82" s="9">
+        <v>0</v>
+      </c>
+      <c r="U82" s="9">
+        <v>0</v>
+      </c>
+      <c r="V82" s="9">
+        <v>0</v>
+      </c>
+      <c r="W82" s="9">
+        <v>0</v>
+      </c>
+      <c r="X82" s="9">
+        <v>0</v>
+      </c>
+      <c r="Y82" s="9">
+        <v>0</v>
+      </c>
+      <c r="Z82" s="9">
+        <v>0</v>
+      </c>
+      <c r="AA82" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83" spans="1:27" x14ac:dyDescent="0.45">
+      <c r="A83" s="4">
+        <v>46203</v>
+      </c>
+      <c r="B83" s="4">
+        <v>46205</v>
+      </c>
+      <c r="C83" s="5">
+        <v>6857</v>
+      </c>
+      <c r="D83" s="9" t="s">
+        <v>458</v>
+      </c>
+      <c r="E83" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="F83" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="G83" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="H83" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="I83" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="J83" s="5">
+        <v>100</v>
+      </c>
+      <c r="K83" s="7">
+        <v>32458.9</v>
+      </c>
+      <c r="L83" s="9">
+        <v>0</v>
+      </c>
+      <c r="M83" s="9">
+        <v>0</v>
+      </c>
+      <c r="N83" s="9">
+        <v>95</v>
+      </c>
+      <c r="O83" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="P83" s="19">
+        <v>-85985</v>
+      </c>
+      <c r="Q83" s="4">
+        <v>46203</v>
+      </c>
+      <c r="R83" s="7">
+        <v>31600</v>
+      </c>
+      <c r="S83" s="9">
+        <v>0</v>
+      </c>
+      <c r="T83" s="9">
+        <v>0</v>
+      </c>
+      <c r="U83" s="9">
+        <v>0</v>
+      </c>
+      <c r="V83" s="9">
+        <v>0</v>
+      </c>
+      <c r="W83" s="9">
+        <v>0</v>
+      </c>
+      <c r="X83" s="9">
+        <v>0</v>
+      </c>
+      <c r="Y83" s="9">
+        <v>95</v>
+      </c>
+      <c r="Z83" s="9">
+        <v>0</v>
+      </c>
+      <c r="AA83" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84" spans="1:27" x14ac:dyDescent="0.45">
+      <c r="A84" s="4">
+        <v>46206</v>
+      </c>
+      <c r="B84" s="4">
+        <v>46210</v>
+      </c>
+      <c r="C84" s="5" t="s">
+        <v>446</v>
+      </c>
+      <c r="D84" s="9" t="s">
+        <v>447</v>
+      </c>
+      <c r="E84" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="F84" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="G84" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="H84" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="I84" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="J84" s="5">
+        <v>100</v>
+      </c>
+      <c r="K84" s="7">
+        <v>73960</v>
+      </c>
+      <c r="L84" s="9">
+        <v>0</v>
+      </c>
+      <c r="M84" s="9">
+        <v>0</v>
+      </c>
+      <c r="N84" s="9">
+        <v>0</v>
+      </c>
+      <c r="O84" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="P84" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q84" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="R84" s="9">
+        <v>0</v>
+      </c>
+      <c r="S84" s="9">
+        <v>0</v>
+      </c>
+      <c r="T84" s="9">
+        <v>0</v>
+      </c>
+      <c r="U84" s="9">
+        <v>0</v>
+      </c>
+      <c r="V84" s="9">
+        <v>0</v>
+      </c>
+      <c r="W84" s="9">
+        <v>0</v>
+      </c>
+      <c r="X84" s="9">
+        <v>0</v>
+      </c>
+      <c r="Y84" s="9">
+        <v>0</v>
+      </c>
+      <c r="Z84" s="9">
+        <v>0</v>
+      </c>
+      <c r="AA84" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85" spans="1:27" x14ac:dyDescent="0.45">
+      <c r="A85" s="4">
+        <v>46206</v>
+      </c>
+      <c r="B85" s="4">
+        <v>46210</v>
+      </c>
+      <c r="C85" s="5" t="s">
+        <v>446</v>
+      </c>
+      <c r="D85" s="9" t="s">
+        <v>447</v>
+      </c>
+      <c r="E85" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="F85" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="G85" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="H85" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="I85" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="J85" s="5">
+        <v>100</v>
+      </c>
+      <c r="K85" s="7">
+        <v>76578</v>
+      </c>
+      <c r="L85" s="9">
+        <v>0</v>
+      </c>
+      <c r="M85" s="9">
+        <v>0</v>
+      </c>
+      <c r="N85" s="9"/>
+      <c r="O85" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="P85" s="20">
+        <v>-261800</v>
+      </c>
+      <c r="Q85" s="4">
+        <v>46206</v>
+      </c>
+      <c r="R85" s="7">
+        <v>73960</v>
+      </c>
+      <c r="S85" s="9">
+        <v>0</v>
+      </c>
+      <c r="T85" s="9">
+        <v>0</v>
+      </c>
+      <c r="U85" s="9">
+        <v>0</v>
+      </c>
+      <c r="V85" s="9">
+        <v>0</v>
+      </c>
+      <c r="W85" s="9">
+        <v>0</v>
+      </c>
+      <c r="X85" s="9">
+        <v>0</v>
+      </c>
+      <c r="Y85" s="9"/>
+      <c r="Z85" s="9">
+        <v>0</v>
+      </c>
+      <c r="AA85" s="9">
         <v>0</v>
       </c>
     </row>

</xml_diff>